<commit_message>
[docs] Recipes 제이슨 수정
</commit_message>
<xml_diff>
--- a/Excel2JSON(win-x64)/excel_files/Data.xlsx
+++ b/Excel2JSON(win-x64)/excel_files/Data.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28816"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E6AAC89C-00BC-4FFA-B7B2-3808DA23F1C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{042C2887-EE4A-4308-B54B-87435F336C13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5040" uniqueCount="981">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5243" uniqueCount="981">
   <si>
     <t>key</t>
   </si>
@@ -2406,7 +2406,7 @@
     <t>쌈장</t>
   </si>
   <si>
-    <t>401, 403, 11</t>
+    <t>110401, 110403, 110011</t>
   </si>
   <si>
     <t>조합 재료</t>
@@ -2415,13 +2415,13 @@
     <t>밀가루 반죽</t>
   </si>
   <si>
-    <t>406, 60</t>
+    <t>110406, 110060</t>
   </si>
   <si>
     <t>고구마 맛탕</t>
   </si>
   <si>
-    <t>124, 11</t>
+    <t>110124, 110011</t>
   </si>
   <si>
     <t>조합 요리</t>
@@ -2430,25 +2430,25 @@
     <t>멸치 볶음</t>
   </si>
   <si>
-    <t>147, 11</t>
+    <t>110147, 110011</t>
   </si>
   <si>
     <t>견과류 멸치 볶음</t>
   </si>
   <si>
-    <t>147, 11, 135</t>
+    <t>110147, 110011, 110135</t>
   </si>
   <si>
     <t>버터 감자</t>
   </si>
   <si>
-    <t>114, 407</t>
+    <t>110114, 1100407</t>
   </si>
   <si>
     <t xml:space="preserve">허니 버터 감자 </t>
   </si>
   <si>
-    <t>114, 407, 11</t>
+    <t>110114, 110407, 110011</t>
   </si>
   <si>
     <t>정어리 회</t>
@@ -24001,11 +24001,11 @@
       <c r="B4" s="9" t="s">
         <v>691</v>
       </c>
-      <c r="C4" s="9">
-        <v>100</v>
-      </c>
-      <c r="D4" s="9">
-        <v>1</v>
+      <c r="C4" s="9" t="s">
+        <v>486</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>425</v>
       </c>
       <c r="E4" s="9">
         <v>1001</v>
@@ -24021,11 +24021,11 @@
       <c r="B5" s="9" t="s">
         <v>693</v>
       </c>
-      <c r="C5" s="9">
-        <v>101</v>
-      </c>
-      <c r="D5" s="9">
-        <v>1</v>
+      <c r="C5" s="9" t="s">
+        <v>487</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>425</v>
       </c>
       <c r="E5" s="9">
         <v>1002</v>
@@ -24041,11 +24041,11 @@
       <c r="B6" s="9" t="s">
         <v>694</v>
       </c>
-      <c r="C6" s="9">
-        <v>102</v>
-      </c>
-      <c r="D6" s="9">
-        <v>2</v>
+      <c r="C6" s="9" t="s">
+        <v>488</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>427</v>
       </c>
       <c r="E6" s="9">
         <v>1001</v>
@@ -24061,11 +24061,11 @@
       <c r="B7" s="9" t="s">
         <v>695</v>
       </c>
-      <c r="C7" s="9">
-        <v>103</v>
-      </c>
-      <c r="D7" s="9">
-        <v>2</v>
+      <c r="C7" s="9" t="s">
+        <v>489</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>427</v>
       </c>
       <c r="E7" s="9">
         <v>1002</v>
@@ -24081,11 +24081,11 @@
       <c r="B8" s="9" t="s">
         <v>696</v>
       </c>
-      <c r="C8" s="9">
-        <v>104</v>
-      </c>
-      <c r="D8" s="9">
-        <v>3</v>
+      <c r="C8" s="9" t="s">
+        <v>490</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>428</v>
       </c>
       <c r="E8" s="9">
         <v>1001</v>
@@ -24101,11 +24101,11 @@
       <c r="B9" s="9" t="s">
         <v>697</v>
       </c>
-      <c r="C9" s="9">
-        <v>105</v>
-      </c>
-      <c r="D9" s="9">
-        <v>3</v>
+      <c r="C9" s="9" t="s">
+        <v>491</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>428</v>
       </c>
       <c r="E9" s="9">
         <v>1003</v>
@@ -24121,11 +24121,11 @@
       <c r="B10" s="9" t="s">
         <v>698</v>
       </c>
-      <c r="C10" s="9">
-        <v>106</v>
-      </c>
-      <c r="D10" s="9">
-        <v>4</v>
+      <c r="C10" s="9" t="s">
+        <v>492</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>429</v>
       </c>
       <c r="E10" s="9">
         <v>1001</v>
@@ -24141,11 +24141,11 @@
       <c r="B11" s="9" t="s">
         <v>699</v>
       </c>
-      <c r="C11" s="9">
-        <v>107</v>
-      </c>
-      <c r="D11" s="9">
-        <v>7</v>
+      <c r="C11" s="9" t="s">
+        <v>493</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>432</v>
       </c>
       <c r="E11" s="9">
         <v>1001</v>
@@ -24161,11 +24161,11 @@
       <c r="B12" s="9" t="s">
         <v>700</v>
       </c>
-      <c r="C12" s="9">
-        <v>108</v>
-      </c>
-      <c r="D12" s="9">
-        <v>7</v>
+      <c r="C12" s="9" t="s">
+        <v>494</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>432</v>
       </c>
       <c r="E12" s="9">
         <v>1006</v>
@@ -24181,11 +24181,11 @@
       <c r="B13" s="9" t="s">
         <v>701</v>
       </c>
-      <c r="C13" s="9">
-        <v>109</v>
-      </c>
-      <c r="D13" s="9">
-        <v>7</v>
+      <c r="C13" s="9" t="s">
+        <v>495</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>432</v>
       </c>
       <c r="E13" s="9">
         <v>1006</v>
@@ -24201,11 +24201,11 @@
       <c r="B14" s="9" t="s">
         <v>702</v>
       </c>
-      <c r="C14" s="9">
-        <v>110</v>
-      </c>
-      <c r="D14" s="9">
-        <v>8</v>
+      <c r="C14" s="9" t="s">
+        <v>496</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>433</v>
       </c>
       <c r="E14" s="9">
         <v>1004</v>
@@ -24221,11 +24221,11 @@
       <c r="B15" s="9" t="s">
         <v>703</v>
       </c>
-      <c r="C15" s="9">
-        <v>111</v>
-      </c>
-      <c r="D15" s="9">
-        <v>8</v>
+      <c r="C15" s="9" t="s">
+        <v>497</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>433</v>
       </c>
       <c r="E15" s="9">
         <v>1005</v>
@@ -24241,11 +24241,11 @@
       <c r="B16" s="9" t="s">
         <v>704</v>
       </c>
-      <c r="C16" s="9">
-        <v>112</v>
-      </c>
-      <c r="D16" s="9">
-        <v>8</v>
+      <c r="C16" s="9" t="s">
+        <v>498</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>433</v>
       </c>
       <c r="E16" s="9">
         <v>1001</v>
@@ -24261,11 +24261,11 @@
       <c r="B17" s="9" t="s">
         <v>705</v>
       </c>
-      <c r="C17" s="9">
-        <v>113</v>
-      </c>
-      <c r="D17" s="9">
-        <v>9</v>
+      <c r="C17" s="9" t="s">
+        <v>499</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>434</v>
       </c>
       <c r="E17" s="9">
         <v>1001</v>
@@ -24281,11 +24281,11 @@
       <c r="B18" s="9" t="s">
         <v>706</v>
       </c>
-      <c r="C18" s="9">
-        <v>114</v>
-      </c>
-      <c r="D18" s="9">
-        <v>9</v>
+      <c r="C18" s="9" t="s">
+        <v>500</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>434</v>
       </c>
       <c r="E18" s="9">
         <v>1006</v>
@@ -24301,11 +24301,11 @@
       <c r="B19" s="9" t="s">
         <v>707</v>
       </c>
-      <c r="C19" s="9">
-        <v>115</v>
-      </c>
-      <c r="D19" s="9">
-        <v>9</v>
+      <c r="C19" s="9" t="s">
+        <v>501</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>434</v>
       </c>
       <c r="E19" s="9">
         <v>1004</v>
@@ -24321,11 +24321,11 @@
       <c r="B20" s="9" t="s">
         <v>708</v>
       </c>
-      <c r="C20" s="9">
-        <v>116</v>
-      </c>
-      <c r="D20" s="9">
-        <v>9</v>
+      <c r="C20" s="9" t="s">
+        <v>502</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>434</v>
       </c>
       <c r="E20" s="9">
         <v>1002</v>
@@ -24341,11 +24341,11 @@
       <c r="B21" s="9" t="s">
         <v>709</v>
       </c>
-      <c r="C21" s="9">
-        <v>117</v>
-      </c>
-      <c r="D21" s="9">
-        <v>10</v>
+      <c r="C21" s="9" t="s">
+        <v>503</v>
+      </c>
+      <c r="D21" s="9" t="s">
+        <v>435</v>
       </c>
       <c r="E21" s="9">
         <v>1004</v>
@@ -24361,11 +24361,11 @@
       <c r="B22" s="9" t="s">
         <v>710</v>
       </c>
-      <c r="C22" s="9">
-        <v>118</v>
-      </c>
-      <c r="D22" s="9">
-        <v>12</v>
+      <c r="C22" s="9" t="s">
+        <v>504</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>437</v>
       </c>
       <c r="E22" s="9">
         <v>1001</v>
@@ -24381,11 +24381,11 @@
       <c r="B23" s="9" t="s">
         <v>711</v>
       </c>
-      <c r="C23" s="9">
-        <v>119</v>
-      </c>
-      <c r="D23" s="9">
-        <v>12</v>
+      <c r="C23" s="9" t="s">
+        <v>505</v>
+      </c>
+      <c r="D23" s="9" t="s">
+        <v>437</v>
       </c>
       <c r="E23" s="9">
         <v>1004</v>
@@ -24401,11 +24401,11 @@
       <c r="B24" s="9" t="s">
         <v>712</v>
       </c>
-      <c r="C24" s="9">
-        <v>120</v>
-      </c>
-      <c r="D24" s="9">
-        <v>12</v>
+      <c r="C24" s="9" t="s">
+        <v>506</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>437</v>
       </c>
       <c r="E24" s="9">
         <v>1003</v>
@@ -24421,11 +24421,11 @@
       <c r="B25" s="9" t="s">
         <v>713</v>
       </c>
-      <c r="C25" s="9">
-        <v>121</v>
-      </c>
-      <c r="D25" s="9">
-        <v>13</v>
+      <c r="C25" s="9" t="s">
+        <v>507</v>
+      </c>
+      <c r="D25" s="9" t="s">
+        <v>438</v>
       </c>
       <c r="E25" s="9">
         <v>1001</v>
@@ -24441,11 +24441,11 @@
       <c r="B26" s="9" t="s">
         <v>714</v>
       </c>
-      <c r="C26" s="9">
-        <v>122</v>
-      </c>
-      <c r="D26" s="9">
-        <v>14</v>
+      <c r="C26" s="9" t="s">
+        <v>508</v>
+      </c>
+      <c r="D26" s="9" t="s">
+        <v>439</v>
       </c>
       <c r="E26" s="9">
         <v>1003</v>
@@ -24461,11 +24461,11 @@
       <c r="B27" s="9" t="s">
         <v>715</v>
       </c>
-      <c r="C27" s="9">
-        <v>123</v>
-      </c>
-      <c r="D27" s="9">
-        <v>15</v>
+      <c r="C27" s="9" t="s">
+        <v>509</v>
+      </c>
+      <c r="D27" s="9" t="s">
+        <v>440</v>
       </c>
       <c r="E27" s="9">
         <v>1001</v>
@@ -24481,11 +24481,11 @@
       <c r="B28" s="9" t="s">
         <v>716</v>
       </c>
-      <c r="C28" s="9">
-        <v>124</v>
-      </c>
-      <c r="D28" s="9">
-        <v>15</v>
+      <c r="C28" s="9" t="s">
+        <v>510</v>
+      </c>
+      <c r="D28" s="9" t="s">
+        <v>440</v>
       </c>
       <c r="E28" s="9">
         <v>1006</v>
@@ -24501,11 +24501,11 @@
       <c r="B29" s="9" t="s">
         <v>717</v>
       </c>
-      <c r="C29" s="9">
-        <v>125</v>
-      </c>
-      <c r="D29" s="9">
-        <v>15</v>
+      <c r="C29" s="9" t="s">
+        <v>511</v>
+      </c>
+      <c r="D29" s="9" t="s">
+        <v>440</v>
       </c>
       <c r="E29" s="9">
         <v>1004</v>
@@ -24521,11 +24521,11 @@
       <c r="B30" s="9" t="s">
         <v>718</v>
       </c>
-      <c r="C30" s="9">
-        <v>126</v>
-      </c>
-      <c r="D30" s="9">
-        <v>15</v>
+      <c r="C30" s="9" t="s">
+        <v>512</v>
+      </c>
+      <c r="D30" s="9" t="s">
+        <v>440</v>
       </c>
       <c r="E30" s="9">
         <v>1002</v>
@@ -24541,11 +24541,11 @@
       <c r="B31" s="9" t="s">
         <v>719</v>
       </c>
-      <c r="C31" s="9">
-        <v>127</v>
-      </c>
-      <c r="D31" s="9">
-        <v>17</v>
+      <c r="C31" s="9" t="s">
+        <v>513</v>
+      </c>
+      <c r="D31" s="9" t="s">
+        <v>442</v>
       </c>
       <c r="E31" s="9">
         <v>1005</v>
@@ -24561,11 +24561,11 @@
       <c r="B32" s="9" t="s">
         <v>720</v>
       </c>
-      <c r="C32" s="9">
-        <v>128</v>
-      </c>
-      <c r="D32" s="9">
-        <v>18</v>
+      <c r="C32" s="9" t="s">
+        <v>514</v>
+      </c>
+      <c r="D32" s="9" t="s">
+        <v>443</v>
       </c>
       <c r="E32" s="9">
         <v>1005</v>
@@ -24581,11 +24581,11 @@
       <c r="B33" s="9" t="s">
         <v>721</v>
       </c>
-      <c r="C33" s="9">
-        <v>129</v>
-      </c>
-      <c r="D33" s="9">
-        <v>18</v>
+      <c r="C33" s="9" t="s">
+        <v>515</v>
+      </c>
+      <c r="D33" s="9" t="s">
+        <v>443</v>
       </c>
       <c r="E33" s="9">
         <v>1002</v>
@@ -24601,11 +24601,11 @@
       <c r="B34" s="9" t="s">
         <v>722</v>
       </c>
-      <c r="C34" s="9">
-        <v>130</v>
-      </c>
-      <c r="D34" s="9">
-        <v>19</v>
+      <c r="C34" s="9" t="s">
+        <v>516</v>
+      </c>
+      <c r="D34" s="9" t="s">
+        <v>444</v>
       </c>
       <c r="E34" s="9">
         <v>1001</v>
@@ -24621,11 +24621,11 @@
       <c r="B35" s="9" t="s">
         <v>723</v>
       </c>
-      <c r="C35" s="9">
-        <v>131</v>
-      </c>
-      <c r="D35" s="9">
-        <v>19</v>
+      <c r="C35" s="9" t="s">
+        <v>517</v>
+      </c>
+      <c r="D35" s="9" t="s">
+        <v>444</v>
       </c>
       <c r="E35" s="9">
         <v>1003</v>
@@ -24641,11 +24641,11 @@
       <c r="B36" s="9" t="s">
         <v>724</v>
       </c>
-      <c r="C36" s="9">
-        <v>132</v>
-      </c>
-      <c r="D36" s="9">
-        <v>20</v>
+      <c r="C36" s="9" t="s">
+        <v>518</v>
+      </c>
+      <c r="D36" s="9" t="s">
+        <v>445</v>
       </c>
       <c r="E36" s="9">
         <v>1001</v>
@@ -24661,11 +24661,11 @@
       <c r="B37" s="9" t="s">
         <v>725</v>
       </c>
-      <c r="C37" s="9">
-        <v>133</v>
-      </c>
-      <c r="D37" s="9">
-        <v>20</v>
+      <c r="C37" s="9" t="s">
+        <v>519</v>
+      </c>
+      <c r="D37" s="9" t="s">
+        <v>445</v>
       </c>
       <c r="E37" s="9">
         <v>1003</v>
@@ -24681,11 +24681,11 @@
       <c r="B38" s="9" t="s">
         <v>726</v>
       </c>
-      <c r="C38" s="9">
-        <v>134</v>
-      </c>
-      <c r="D38" s="9">
-        <v>21</v>
+      <c r="C38" s="9" t="s">
+        <v>520</v>
+      </c>
+      <c r="D38" s="9" t="s">
+        <v>446</v>
       </c>
       <c r="E38" s="9">
         <v>1002</v>
@@ -24701,11 +24701,11 @@
       <c r="B39" s="9" t="s">
         <v>727</v>
       </c>
-      <c r="C39" s="9">
-        <v>135</v>
-      </c>
-      <c r="D39" s="9">
-        <v>21</v>
+      <c r="C39" s="9" t="s">
+        <v>521</v>
+      </c>
+      <c r="D39" s="9" t="s">
+        <v>446</v>
       </c>
       <c r="E39" s="9">
         <v>1001</v>
@@ -24721,11 +24721,11 @@
       <c r="B40" s="9" t="s">
         <v>728</v>
       </c>
-      <c r="C40" s="9">
-        <v>136</v>
-      </c>
-      <c r="D40" s="9">
-        <v>22</v>
+      <c r="C40" s="9" t="s">
+        <v>522</v>
+      </c>
+      <c r="D40" s="9" t="s">
+        <v>447</v>
       </c>
       <c r="E40" s="9">
         <v>1001</v>
@@ -24741,11 +24741,11 @@
       <c r="B41" s="9" t="s">
         <v>729</v>
       </c>
-      <c r="C41" s="9">
-        <v>137</v>
-      </c>
-      <c r="D41" s="9">
-        <v>23</v>
+      <c r="C41" s="9" t="s">
+        <v>523</v>
+      </c>
+      <c r="D41" s="9" t="s">
+        <v>448</v>
       </c>
       <c r="E41" s="9">
         <v>1001</v>
@@ -24761,11 +24761,11 @@
       <c r="B42" s="9" t="s">
         <v>730</v>
       </c>
-      <c r="C42" s="9">
-        <v>138</v>
-      </c>
-      <c r="D42" s="9">
-        <v>24</v>
+      <c r="C42" s="9" t="s">
+        <v>524</v>
+      </c>
+      <c r="D42" s="9" t="s">
+        <v>449</v>
       </c>
       <c r="E42" s="9">
         <v>1001</v>
@@ -24781,11 +24781,11 @@
       <c r="B43" s="9" t="s">
         <v>731</v>
       </c>
-      <c r="C43" s="9">
-        <v>139</v>
-      </c>
-      <c r="D43" s="9">
-        <v>24</v>
+      <c r="C43" s="9" t="s">
+        <v>525</v>
+      </c>
+      <c r="D43" s="9" t="s">
+        <v>449</v>
       </c>
       <c r="E43" s="9">
         <v>1003</v>
@@ -24801,11 +24801,11 @@
       <c r="B44" s="9" t="s">
         <v>732</v>
       </c>
-      <c r="C44" s="9">
-        <v>140</v>
-      </c>
-      <c r="D44" s="9">
-        <v>27</v>
+      <c r="C44" s="9" t="s">
+        <v>526</v>
+      </c>
+      <c r="D44" s="9" t="s">
+        <v>452</v>
       </c>
       <c r="E44" s="9">
         <v>1001</v>
@@ -24821,11 +24821,11 @@
       <c r="B45" s="9" t="s">
         <v>733</v>
       </c>
-      <c r="C45" s="9">
-        <v>141</v>
-      </c>
-      <c r="D45" s="9">
-        <v>27</v>
+      <c r="C45" s="9" t="s">
+        <v>527</v>
+      </c>
+      <c r="D45" s="9" t="s">
+        <v>452</v>
       </c>
       <c r="E45" s="9">
         <v>1001</v>
@@ -24841,11 +24841,11 @@
       <c r="B46" s="9" t="s">
         <v>734</v>
       </c>
-      <c r="C46" s="9">
-        <v>142</v>
-      </c>
-      <c r="D46" s="9">
-        <v>28</v>
+      <c r="C46" s="9" t="s">
+        <v>528</v>
+      </c>
+      <c r="D46" s="9" t="s">
+        <v>453</v>
       </c>
       <c r="E46" s="9">
         <v>1004</v>
@@ -24861,11 +24861,11 @@
       <c r="B47" s="9" t="s">
         <v>735</v>
       </c>
-      <c r="C47" s="9">
-        <v>143</v>
-      </c>
-      <c r="D47" s="9">
-        <v>32</v>
+      <c r="C47" s="9" t="s">
+        <v>529</v>
+      </c>
+      <c r="D47" s="9" t="s">
+        <v>457</v>
       </c>
       <c r="E47" s="9">
         <v>1001</v>
@@ -24881,11 +24881,11 @@
       <c r="B48" s="9" t="s">
         <v>736</v>
       </c>
-      <c r="C48" s="9">
-        <v>144</v>
-      </c>
-      <c r="D48" s="9">
-        <v>32</v>
+      <c r="C48" s="9" t="s">
+        <v>530</v>
+      </c>
+      <c r="D48" s="9" t="s">
+        <v>457</v>
       </c>
       <c r="E48" s="9">
         <v>1001</v>
@@ -24901,11 +24901,11 @@
       <c r="B49" s="9" t="s">
         <v>737</v>
       </c>
-      <c r="C49" s="9">
-        <v>145</v>
-      </c>
-      <c r="D49" s="9">
-        <v>32</v>
+      <c r="C49" s="9" t="s">
+        <v>531</v>
+      </c>
+      <c r="D49" s="9" t="s">
+        <v>457</v>
       </c>
       <c r="E49" s="9">
         <v>1006</v>
@@ -24921,11 +24921,11 @@
       <c r="B50" s="9" t="s">
         <v>738</v>
       </c>
-      <c r="C50" s="9">
-        <v>146</v>
-      </c>
-      <c r="D50" s="9">
-        <v>33</v>
+      <c r="C50" s="9" t="s">
+        <v>532</v>
+      </c>
+      <c r="D50" s="9" t="s">
+        <v>458</v>
       </c>
       <c r="E50" s="9">
         <v>1001</v>
@@ -24941,11 +24941,11 @@
       <c r="B51" s="9" t="s">
         <v>739</v>
       </c>
-      <c r="C51" s="9">
-        <v>147</v>
-      </c>
-      <c r="D51" s="9">
-        <v>33</v>
+      <c r="C51" s="9" t="s">
+        <v>533</v>
+      </c>
+      <c r="D51" s="9" t="s">
+        <v>458</v>
       </c>
       <c r="E51" s="9">
         <v>1006</v>
@@ -24961,11 +24961,11 @@
       <c r="B52" s="9" t="s">
         <v>740</v>
       </c>
-      <c r="C52" s="9">
-        <v>148</v>
-      </c>
-      <c r="D52" s="9">
-        <v>34</v>
+      <c r="C52" s="9" t="s">
+        <v>534</v>
+      </c>
+      <c r="D52" s="9" t="s">
+        <v>459</v>
       </c>
       <c r="E52" s="9">
         <v>1004</v>
@@ -24981,11 +24981,11 @@
       <c r="B53" s="9" t="s">
         <v>741</v>
       </c>
-      <c r="C53" s="9">
-        <v>149</v>
-      </c>
-      <c r="D53" s="9">
-        <v>35</v>
+      <c r="C53" s="9" t="s">
+        <v>535</v>
+      </c>
+      <c r="D53" s="9" t="s">
+        <v>460</v>
       </c>
       <c r="E53" s="9">
         <v>1004</v>
@@ -25001,11 +25001,11 @@
       <c r="B54" s="9" t="s">
         <v>742</v>
       </c>
-      <c r="C54" s="9">
-        <v>150</v>
-      </c>
-      <c r="D54" s="9">
-        <v>36</v>
+      <c r="C54" s="9" t="s">
+        <v>536</v>
+      </c>
+      <c r="D54" s="9" t="s">
+        <v>461</v>
       </c>
       <c r="E54" s="9">
         <v>1001</v>
@@ -25021,11 +25021,11 @@
       <c r="B55" s="9" t="s">
         <v>743</v>
       </c>
-      <c r="C55" s="9">
-        <v>151</v>
-      </c>
-      <c r="D55" s="9">
-        <v>36</v>
+      <c r="C55" s="9" t="s">
+        <v>537</v>
+      </c>
+      <c r="D55" s="9" t="s">
+        <v>461</v>
       </c>
       <c r="E55" s="9">
         <v>1001</v>
@@ -25041,11 +25041,11 @@
       <c r="B56" s="9" t="s">
         <v>744</v>
       </c>
-      <c r="C56" s="9">
-        <v>152</v>
-      </c>
-      <c r="D56" s="9">
-        <v>36</v>
+      <c r="C56" s="9" t="s">
+        <v>538</v>
+      </c>
+      <c r="D56" s="9" t="s">
+        <v>461</v>
       </c>
       <c r="E56" s="9">
         <v>1006</v>
@@ -25061,11 +25061,11 @@
       <c r="B57" s="9" t="s">
         <v>745</v>
       </c>
-      <c r="C57" s="9">
-        <v>153</v>
-      </c>
-      <c r="D57" s="9">
-        <v>37</v>
+      <c r="C57" s="9" t="s">
+        <v>539</v>
+      </c>
+      <c r="D57" s="9" t="s">
+        <v>462</v>
       </c>
       <c r="E57" s="9">
         <v>1001</v>
@@ -25081,11 +25081,11 @@
       <c r="B58" s="9" t="s">
         <v>746</v>
       </c>
-      <c r="C58" s="9">
-        <v>154</v>
-      </c>
-      <c r="D58" s="9">
-        <v>39</v>
+      <c r="C58" s="9" t="s">
+        <v>540</v>
+      </c>
+      <c r="D58" s="9" t="s">
+        <v>464</v>
       </c>
       <c r="E58" s="9">
         <v>1001</v>
@@ -25101,11 +25101,11 @@
       <c r="B59" s="9" t="s">
         <v>747</v>
       </c>
-      <c r="C59" s="9">
-        <v>155</v>
-      </c>
-      <c r="D59" s="9">
-        <v>39</v>
+      <c r="C59" s="9" t="s">
+        <v>541</v>
+      </c>
+      <c r="D59" s="9" t="s">
+        <v>464</v>
       </c>
       <c r="E59" s="9">
         <v>1001</v>
@@ -25121,11 +25121,11 @@
       <c r="B60" s="9" t="s">
         <v>748</v>
       </c>
-      <c r="C60" s="9">
-        <v>156</v>
-      </c>
-      <c r="D60" s="9">
-        <v>40</v>
+      <c r="C60" s="9" t="s">
+        <v>542</v>
+      </c>
+      <c r="D60" s="9" t="s">
+        <v>465</v>
       </c>
       <c r="E60" s="9">
         <v>1005</v>
@@ -25141,11 +25141,11 @@
       <c r="B61" s="9" t="s">
         <v>749</v>
       </c>
-      <c r="C61" s="9">
-        <v>157</v>
-      </c>
-      <c r="D61" s="9">
-        <v>41</v>
+      <c r="C61" s="9" t="s">
+        <v>543</v>
+      </c>
+      <c r="D61" s="9" t="s">
+        <v>466</v>
       </c>
       <c r="E61" s="9">
         <v>1001</v>
@@ -25161,11 +25161,11 @@
       <c r="B62" s="9" t="s">
         <v>750</v>
       </c>
-      <c r="C62" s="9">
-        <v>158</v>
-      </c>
-      <c r="D62" s="9">
-        <v>42</v>
+      <c r="C62" s="9" t="s">
+        <v>544</v>
+      </c>
+      <c r="D62" s="9" t="s">
+        <v>467</v>
       </c>
       <c r="E62" s="9">
         <v>1001</v>
@@ -25181,11 +25181,11 @@
       <c r="B63" s="9" t="s">
         <v>751</v>
       </c>
-      <c r="C63" s="9">
-        <v>159</v>
-      </c>
-      <c r="D63" s="9">
-        <v>42</v>
+      <c r="C63" s="9" t="s">
+        <v>545</v>
+      </c>
+      <c r="D63" s="9" t="s">
+        <v>467</v>
       </c>
       <c r="E63" s="9">
         <v>1001</v>
@@ -25201,11 +25201,11 @@
       <c r="B64" s="9" t="s">
         <v>752</v>
       </c>
-      <c r="C64" s="9">
-        <v>160</v>
-      </c>
-      <c r="D64" s="9">
-        <v>42</v>
+      <c r="C64" s="9" t="s">
+        <v>546</v>
+      </c>
+      <c r="D64" s="9" t="s">
+        <v>467</v>
       </c>
       <c r="E64" s="9">
         <v>1006</v>
@@ -25221,11 +25221,11 @@
       <c r="B65" s="9" t="s">
         <v>753</v>
       </c>
-      <c r="C65" s="9">
-        <v>161</v>
-      </c>
-      <c r="D65" s="9">
-        <v>44</v>
+      <c r="C65" s="9" t="s">
+        <v>547</v>
+      </c>
+      <c r="D65" s="9" t="s">
+        <v>469</v>
       </c>
       <c r="E65" s="9">
         <v>1001</v>
@@ -25241,11 +25241,11 @@
       <c r="B66" s="9" t="s">
         <v>754</v>
       </c>
-      <c r="C66" s="9">
-        <v>162</v>
-      </c>
-      <c r="D66" s="9">
-        <v>44</v>
+      <c r="C66" s="9" t="s">
+        <v>548</v>
+      </c>
+      <c r="D66" s="9" t="s">
+        <v>469</v>
       </c>
       <c r="E66" s="9">
         <v>1001</v>
@@ -25261,11 +25261,11 @@
       <c r="B67" s="9" t="s">
         <v>755</v>
       </c>
-      <c r="C67" s="9">
-        <v>163</v>
-      </c>
-      <c r="D67" s="9">
-        <v>44</v>
+      <c r="C67" s="9" t="s">
+        <v>549</v>
+      </c>
+      <c r="D67" s="9" t="s">
+        <v>469</v>
       </c>
       <c r="E67" s="9">
         <v>1001</v>
@@ -25281,11 +25281,11 @@
       <c r="B68" s="9" t="s">
         <v>756</v>
       </c>
-      <c r="C68" s="9">
-        <v>164</v>
-      </c>
-      <c r="D68" s="9">
-        <v>44</v>
+      <c r="C68" s="9" t="s">
+        <v>550</v>
+      </c>
+      <c r="D68" s="9" t="s">
+        <v>469</v>
       </c>
       <c r="E68" s="9">
         <v>1005</v>
@@ -25301,11 +25301,11 @@
       <c r="B69" s="9" t="s">
         <v>757</v>
       </c>
-      <c r="C69" s="9">
-        <v>165</v>
-      </c>
-      <c r="D69" s="9">
-        <v>44</v>
+      <c r="C69" s="9" t="s">
+        <v>551</v>
+      </c>
+      <c r="D69" s="9" t="s">
+        <v>469</v>
       </c>
       <c r="E69" s="9">
         <v>1006</v>
@@ -25321,11 +25321,11 @@
       <c r="B70" s="9" t="s">
         <v>758</v>
       </c>
-      <c r="C70" s="9">
-        <v>166</v>
-      </c>
-      <c r="D70" s="9">
-        <v>45</v>
+      <c r="C70" s="9" t="s">
+        <v>552</v>
+      </c>
+      <c r="D70" s="9" t="s">
+        <v>470</v>
       </c>
       <c r="E70" s="9">
         <v>1001</v>
@@ -25341,11 +25341,11 @@
       <c r="B71" s="9" t="s">
         <v>759</v>
       </c>
-      <c r="C71" s="9">
-        <v>167</v>
-      </c>
-      <c r="D71" s="9">
-        <v>45</v>
+      <c r="C71" s="9" t="s">
+        <v>553</v>
+      </c>
+      <c r="D71" s="9" t="s">
+        <v>470</v>
       </c>
       <c r="E71" s="9">
         <v>1001</v>
@@ -25361,11 +25361,11 @@
       <c r="B72" s="9" t="s">
         <v>760</v>
       </c>
-      <c r="C72" s="9">
-        <v>168</v>
-      </c>
-      <c r="D72" s="9">
-        <v>45</v>
+      <c r="C72" s="9" t="s">
+        <v>554</v>
+      </c>
+      <c r="D72" s="9" t="s">
+        <v>470</v>
       </c>
       <c r="E72" s="9">
         <v>1005</v>
@@ -25381,11 +25381,11 @@
       <c r="B73" s="9" t="s">
         <v>761</v>
       </c>
-      <c r="C73" s="9">
-        <v>169</v>
-      </c>
-      <c r="D73" s="9">
-        <v>46</v>
+      <c r="C73" s="9" t="s">
+        <v>555</v>
+      </c>
+      <c r="D73" s="9" t="s">
+        <v>471</v>
       </c>
       <c r="E73" s="9">
         <v>1001</v>
@@ -25401,11 +25401,11 @@
       <c r="B74" s="9" t="s">
         <v>762</v>
       </c>
-      <c r="C74" s="9">
-        <v>170</v>
-      </c>
-      <c r="D74" s="9">
-        <v>46</v>
+      <c r="C74" s="9" t="s">
+        <v>556</v>
+      </c>
+      <c r="D74" s="9" t="s">
+        <v>471</v>
       </c>
       <c r="E74" s="9">
         <v>1005</v>
@@ -25421,11 +25421,11 @@
       <c r="B75" s="9" t="s">
         <v>763</v>
       </c>
-      <c r="C75" s="9">
-        <v>171</v>
-      </c>
-      <c r="D75" s="9">
-        <v>46</v>
+      <c r="C75" s="9" t="s">
+        <v>557</v>
+      </c>
+      <c r="D75" s="9" t="s">
+        <v>471</v>
       </c>
       <c r="E75" s="9">
         <v>1006</v>
@@ -25441,11 +25441,11 @@
       <c r="B76" s="9" t="s">
         <v>764</v>
       </c>
-      <c r="C76" s="9">
-        <v>172</v>
-      </c>
-      <c r="D76" s="9">
-        <v>47</v>
+      <c r="C76" s="9" t="s">
+        <v>558</v>
+      </c>
+      <c r="D76" s="9" t="s">
+        <v>472</v>
       </c>
       <c r="E76" s="9">
         <v>1001</v>
@@ -25461,11 +25461,11 @@
       <c r="B77" s="9" t="s">
         <v>765</v>
       </c>
-      <c r="C77" s="9">
-        <v>173</v>
-      </c>
-      <c r="D77" s="9">
-        <v>47</v>
+      <c r="C77" s="9" t="s">
+        <v>559</v>
+      </c>
+      <c r="D77" s="9" t="s">
+        <v>472</v>
       </c>
       <c r="E77" s="9">
         <v>1001</v>
@@ -25481,11 +25481,11 @@
       <c r="B78" s="9" t="s">
         <v>766</v>
       </c>
-      <c r="C78" s="9">
-        <v>174</v>
-      </c>
-      <c r="D78" s="9">
-        <v>47</v>
+      <c r="C78" s="9" t="s">
+        <v>560</v>
+      </c>
+      <c r="D78" s="9" t="s">
+        <v>472</v>
       </c>
       <c r="E78" s="9">
         <v>1005</v>
@@ -25501,11 +25501,11 @@
       <c r="B79" s="9" t="s">
         <v>767</v>
       </c>
-      <c r="C79" s="9">
-        <v>175</v>
-      </c>
-      <c r="D79" s="9">
-        <v>47</v>
+      <c r="C79" s="9" t="s">
+        <v>561</v>
+      </c>
+      <c r="D79" s="9" t="s">
+        <v>472</v>
       </c>
       <c r="E79" s="9">
         <v>1001</v>
@@ -25521,11 +25521,11 @@
       <c r="B80" s="9" t="s">
         <v>768</v>
       </c>
-      <c r="C80" s="9">
-        <v>176</v>
-      </c>
-      <c r="D80" s="9">
-        <v>48</v>
+      <c r="C80" s="9" t="s">
+        <v>563</v>
+      </c>
+      <c r="D80" s="9" t="s">
+        <v>473</v>
       </c>
       <c r="E80" s="9">
         <v>1001</v>
@@ -25541,11 +25541,11 @@
       <c r="B81" s="9" t="s">
         <v>769</v>
       </c>
-      <c r="C81" s="9">
-        <v>177</v>
-      </c>
-      <c r="D81" s="9">
-        <v>48</v>
+      <c r="C81" s="9" t="s">
+        <v>564</v>
+      </c>
+      <c r="D81" s="9" t="s">
+        <v>473</v>
       </c>
       <c r="E81" s="9">
         <v>1001</v>
@@ -25561,11 +25561,11 @@
       <c r="B82" s="9" t="s">
         <v>770</v>
       </c>
-      <c r="C82" s="9">
-        <v>178</v>
-      </c>
-      <c r="D82" s="9">
-        <v>48</v>
+      <c r="C82" s="9" t="s">
+        <v>566</v>
+      </c>
+      <c r="D82" s="9" t="s">
+        <v>473</v>
       </c>
       <c r="E82" s="9">
         <v>1005</v>
@@ -25581,11 +25581,11 @@
       <c r="B83" s="9" t="s">
         <v>771</v>
       </c>
-      <c r="C83" s="9">
-        <v>179</v>
-      </c>
-      <c r="D83" s="9">
-        <v>50</v>
+      <c r="C83" s="9" t="s">
+        <v>567</v>
+      </c>
+      <c r="D83" s="9" t="s">
+        <v>475</v>
       </c>
       <c r="E83" s="9">
         <v>1001</v>
@@ -25601,11 +25601,11 @@
       <c r="B84" s="9" t="s">
         <v>772</v>
       </c>
-      <c r="C84" s="9">
-        <v>180</v>
-      </c>
-      <c r="D84" s="9">
-        <v>50</v>
+      <c r="C84" s="9" t="s">
+        <v>568</v>
+      </c>
+      <c r="D84" s="9" t="s">
+        <v>475</v>
       </c>
       <c r="E84" s="9">
         <v>1001</v>
@@ -25621,11 +25621,11 @@
       <c r="B85" s="9" t="s">
         <v>773</v>
       </c>
-      <c r="C85" s="9">
-        <v>181</v>
-      </c>
-      <c r="D85" s="9">
-        <v>50</v>
+      <c r="C85" s="9" t="s">
+        <v>569</v>
+      </c>
+      <c r="D85" s="9" t="s">
+        <v>475</v>
       </c>
       <c r="E85" s="9">
         <v>1005</v>
@@ -25641,11 +25641,11 @@
       <c r="B86" s="9" t="s">
         <v>774</v>
       </c>
-      <c r="C86" s="9">
-        <v>182</v>
-      </c>
-      <c r="D86" s="9">
-        <v>50</v>
+      <c r="C86" s="9" t="s">
+        <v>570</v>
+      </c>
+      <c r="D86" s="9" t="s">
+        <v>475</v>
       </c>
       <c r="E86" s="9">
         <v>1001</v>
@@ -25661,11 +25661,11 @@
       <c r="B87" s="9" t="s">
         <v>775</v>
       </c>
-      <c r="C87" s="9">
-        <v>183</v>
-      </c>
-      <c r="D87" s="9">
-        <v>52</v>
+      <c r="C87" s="9" t="s">
+        <v>571</v>
+      </c>
+      <c r="D87" s="9" t="s">
+        <v>477</v>
       </c>
       <c r="E87" s="9">
         <v>1005</v>
@@ -25681,11 +25681,11 @@
       <c r="B88" s="9" t="s">
         <v>776</v>
       </c>
-      <c r="C88" s="9">
-        <v>184</v>
-      </c>
-      <c r="D88" s="9">
-        <v>52</v>
+      <c r="C88" s="9" t="s">
+        <v>572</v>
+      </c>
+      <c r="D88" s="9" t="s">
+        <v>477</v>
       </c>
       <c r="E88" s="9">
         <v>1006</v>
@@ -25701,11 +25701,11 @@
       <c r="B89" s="9" t="s">
         <v>777</v>
       </c>
-      <c r="C89" s="9">
-        <v>185</v>
-      </c>
-      <c r="D89" s="9">
-        <v>53</v>
+      <c r="C89" s="9" t="s">
+        <v>573</v>
+      </c>
+      <c r="D89" s="9" t="s">
+        <v>478</v>
       </c>
       <c r="E89" s="9">
         <v>1005</v>
@@ -25721,11 +25721,11 @@
       <c r="B90" s="9" t="s">
         <v>778</v>
       </c>
-      <c r="C90" s="9">
-        <v>186</v>
-      </c>
-      <c r="D90" s="9">
-        <v>53</v>
+      <c r="C90" s="9" t="s">
+        <v>574</v>
+      </c>
+      <c r="D90" s="9" t="s">
+        <v>478</v>
       </c>
       <c r="E90" s="9">
         <v>1006</v>
@@ -25741,11 +25741,11 @@
       <c r="B91" s="9" t="s">
         <v>779</v>
       </c>
-      <c r="C91" s="9">
-        <v>187</v>
-      </c>
-      <c r="D91" s="9">
-        <v>54</v>
+      <c r="C91" s="9" t="s">
+        <v>575</v>
+      </c>
+      <c r="D91" s="9" t="s">
+        <v>479</v>
       </c>
       <c r="E91" s="9">
         <v>1005</v>
@@ -25761,11 +25761,11 @@
       <c r="B92" s="9" t="s">
         <v>780</v>
       </c>
-      <c r="C92" s="9">
-        <v>188</v>
-      </c>
-      <c r="D92" s="9">
-        <v>56</v>
+      <c r="C92" s="9" t="s">
+        <v>576</v>
+      </c>
+      <c r="D92" s="9" t="s">
+        <v>481</v>
       </c>
       <c r="E92" s="9">
         <v>1001</v>
@@ -25781,11 +25781,11 @@
       <c r="B93" s="9" t="s">
         <v>781</v>
       </c>
-      <c r="C93" s="9">
-        <v>189</v>
-      </c>
-      <c r="D93" s="9">
-        <v>56</v>
+      <c r="C93" s="9" t="s">
+        <v>577</v>
+      </c>
+      <c r="D93" s="9" t="s">
+        <v>481</v>
       </c>
       <c r="E93" s="9">
         <v>1001</v>
@@ -25801,11 +25801,11 @@
       <c r="B94" s="9" t="s">
         <v>782</v>
       </c>
-      <c r="C94" s="9">
-        <v>190</v>
-      </c>
-      <c r="D94" s="9">
-        <v>57</v>
+      <c r="C94" s="9" t="s">
+        <v>578</v>
+      </c>
+      <c r="D94" s="9" t="s">
+        <v>482</v>
       </c>
       <c r="E94" s="9">
         <v>1001</v>
@@ -25821,11 +25821,11 @@
       <c r="B95" s="9" t="s">
         <v>783</v>
       </c>
-      <c r="C95" s="9">
-        <v>191</v>
-      </c>
-      <c r="D95" s="9">
-        <v>57</v>
+      <c r="C95" s="9" t="s">
+        <v>579</v>
+      </c>
+      <c r="D95" s="9" t="s">
+        <v>482</v>
       </c>
       <c r="E95" s="9">
         <v>1003</v>
@@ -25841,11 +25841,11 @@
       <c r="B96" s="9" t="s">
         <v>784</v>
       </c>
-      <c r="C96" s="9">
-        <v>192</v>
-      </c>
-      <c r="D96" s="9">
-        <v>58</v>
+      <c r="C96" s="9" t="s">
+        <v>580</v>
+      </c>
+      <c r="D96" s="9" t="s">
+        <v>483</v>
       </c>
       <c r="E96" s="9">
         <v>1001</v>
@@ -25861,11 +25861,11 @@
       <c r="B97" s="9" t="s">
         <v>785</v>
       </c>
-      <c r="C97" s="9">
-        <v>193</v>
-      </c>
-      <c r="D97" s="9">
-        <v>58</v>
+      <c r="C97" s="9" t="s">
+        <v>581</v>
+      </c>
+      <c r="D97" s="9" t="s">
+        <v>483</v>
       </c>
       <c r="E97" s="9">
         <v>1003</v>
@@ -25881,11 +25881,11 @@
       <c r="B98" s="9" t="s">
         <v>786</v>
       </c>
-      <c r="C98" s="9">
-        <v>194</v>
-      </c>
-      <c r="D98" s="9">
-        <v>405</v>
+      <c r="C98" s="9" t="s">
+        <v>582</v>
+      </c>
+      <c r="D98" s="9" t="s">
+        <v>590</v>
       </c>
       <c r="E98" s="9">
         <v>1004</v>
@@ -25901,11 +25901,11 @@
       <c r="B99" s="9" t="s">
         <v>787</v>
       </c>
-      <c r="C99" s="9">
-        <v>195</v>
-      </c>
-      <c r="D99" s="9">
-        <v>404</v>
+      <c r="C99" s="9" t="s">
+        <v>583</v>
+      </c>
+      <c r="D99" s="9" t="s">
+        <v>589</v>
       </c>
       <c r="E99" s="9">
         <v>1004</v>
@@ -25921,8 +25921,8 @@
       <c r="B100" s="9" t="s">
         <v>788</v>
       </c>
-      <c r="C100" s="9">
-        <v>194</v>
+      <c r="C100" s="9" t="s">
+        <v>582</v>
       </c>
       <c r="D100" s="9" t="s">
         <v>789</v>
@@ -25941,8 +25941,8 @@
       <c r="B101" s="9" t="s">
         <v>791</v>
       </c>
-      <c r="C101" s="9">
-        <v>196</v>
+      <c r="C101" s="9" t="s">
+        <v>584</v>
       </c>
       <c r="D101" s="9" t="s">
         <v>792</v>
@@ -25961,8 +25961,8 @@
       <c r="B102" s="9" t="s">
         <v>793</v>
       </c>
-      <c r="C102" s="9">
-        <v>501</v>
+      <c r="C102" s="9" t="s">
+        <v>593</v>
       </c>
       <c r="D102" s="9" t="s">
         <v>794</v>
@@ -25981,8 +25981,8 @@
       <c r="B103" s="9" t="s">
         <v>796</v>
       </c>
-      <c r="C103" s="9">
-        <v>502</v>
+      <c r="C103" s="9" t="s">
+        <v>594</v>
       </c>
       <c r="D103" s="9" t="s">
         <v>797</v>
@@ -26001,8 +26001,8 @@
       <c r="B104" s="9" t="s">
         <v>798</v>
       </c>
-      <c r="C104" s="9">
-        <v>503</v>
+      <c r="C104" s="9" t="s">
+        <v>595</v>
       </c>
       <c r="D104" s="9" t="s">
         <v>799</v>
@@ -26021,8 +26021,8 @@
       <c r="B105" s="9" t="s">
         <v>800</v>
       </c>
-      <c r="C105" s="9">
-        <v>504</v>
+      <c r="C105" s="9" t="s">
+        <v>596</v>
       </c>
       <c r="D105" s="9" t="s">
         <v>801</v>
@@ -26041,8 +26041,8 @@
       <c r="B106" s="9" t="s">
         <v>802</v>
       </c>
-      <c r="C106" s="9">
-        <v>505</v>
+      <c r="C106" s="9" t="s">
+        <v>597</v>
       </c>
       <c r="D106" s="9" t="s">
         <v>803</v>
@@ -26061,11 +26061,11 @@
       <c r="B107" s="9" t="s">
         <v>804</v>
       </c>
-      <c r="C107" s="9">
-        <v>506</v>
-      </c>
-      <c r="D107" s="9">
-        <v>144</v>
+      <c r="C107" s="9" t="s">
+        <v>600</v>
+      </c>
+      <c r="D107" s="9" t="s">
+        <v>530</v>
       </c>
       <c r="E107" s="9">
         <v>1008</v>
@@ -26081,11 +26081,11 @@
       <c r="B108" s="9" t="s">
         <v>805</v>
       </c>
-      <c r="C108" s="9">
-        <v>507</v>
-      </c>
-      <c r="D108" s="9">
-        <v>145</v>
+      <c r="C108" s="9" t="s">
+        <v>601</v>
+      </c>
+      <c r="D108" s="9" t="s">
+        <v>531</v>
       </c>
       <c r="E108" s="9">
         <v>1008</v>

</xml_diff>